<commit_message>
Update site data and import roster script for improved functionality
</commit_message>
<xml_diff>
--- a/assets/Strategy & Operations Service Lines v2.xlsx
+++ b/assets/Strategy & Operations Service Lines v2.xlsx
@@ -14116,6 +14116,9 @@
       <c r="D321" s="16"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A140:A183">
+    <cfRule type="duplicateValues" priority="383"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A184:C1048576 A1:C139">
     <cfRule type="duplicateValues" priority="4"/>
   </conditionalFormatting>
@@ -14124,9 +14127,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="N1:N133">
     <cfRule type="duplicateValues" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A140:A183">
-    <cfRule type="duplicateValues" priority="383"/>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" display="https://www.linkedin.com/in/michaelgordon20/" xr:uid="{AA46F59F-9FA5-4C8A-B775-11B0A35DA450}"/>
@@ -14453,6 +14453,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="18c801aa-b08e-4147-8d71-4a4146fc5f82">
@@ -14461,15 +14470,6 @@
     <TaxCatchAll xmlns="964029ae-dec3-475d-8111-d2dd7b517bae" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14660,6 +14660,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898626DD-6B53-4F3D-BC27-4B5A8D32B3B3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA9E554-1ADE-46CE-8803-AC258E13C25F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -14672,14 +14680,6 @@
     <ds:schemaRef ds:uri="964029ae-dec3-475d-8111-d2dd7b517bae"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898626DD-6B53-4F3D-BC27-4B5A8D32B3B3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>